<commit_message>
bug fix and changed opening balance flow
</commit_message>
<xml_diff>
--- a/public/assets/templates/bulk_purchase_order.xlsx
+++ b/public/assets/templates/bulk_purchase_order.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Category</t>
   </si>
@@ -29,6 +29,12 @@
   </si>
   <si>
     <t>Quantity</t>
+  </si>
+  <si>
+    <t>Price Per Unit</t>
+  </si>
+  <si>
+    <t>Tax</t>
   </si>
   <si>
     <t>Discount</t>
@@ -41,7 +47,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -53,13 +59,24 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCFCFD"/>
+        <bgColor rgb="FFFCFCFD"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -68,12 +85,15 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -296,8 +316,8 @@
     <col customWidth="1" min="2" max="2" width="24.75"/>
     <col customWidth="1" min="3" max="3" width="25.13"/>
     <col customWidth="1" min="4" max="5" width="25.75"/>
-    <col customWidth="1" min="6" max="7" width="25.38"/>
-    <col customWidth="1" min="8" max="8" width="25.75"/>
+    <col customWidth="1" min="6" max="9" width="25.38"/>
+    <col customWidth="1" min="10" max="10" width="25.75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -319,11 +339,17 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>